<commit_message>
Added keyword-driven framework changes and .gitignore
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/LoginData.xlsx
+++ b/src/test/resources/testdata/LoginData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joshi\eclipse-workspace\Jarvis\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35497728-584A-42F5-9CC0-D328C451CFAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11027CCF-438D-4F9A-A385-04CBF59242A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{EAE6DA33-F364-463F-85B1-05798DBEF51C}"/>
   </bookViews>
@@ -27,8 +27,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -100,13 +98,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -441,17 +436,18 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A2" s="3" t="s">
+    <row r="2" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" t="s">
         <v>3</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" display="mailto:vaceyi3307@pazard.com" xr:uid="{CEEE3E60-1B76-4B86-9CD2-15880505CBFD}"/>
+    <hyperlink ref="A2" r:id="rId1" xr:uid="{CEEE3E60-1B76-4B86-9CD2-15880505CBFD}"/>
+    <hyperlink ref="B2" r:id="rId2" xr:uid="{E4498525-CA1B-483A-88E8-F4BBFEBDB590}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>